<commit_message>
fix: prevent building-tabs-wrapper from shrinking in flex layout
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-The Monet 第1期.xlsx
+++ b/files/九龙-九龙塘-The Monet 第1期.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="销控汇总明细" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2座 销控表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3座 销控表" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,65 +39,8 @@
       <name val="Microsoft YaHei"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <color rgb="007F7F7F"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="007F7F7F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="00004D00"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="00004D00"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <color rgb="00002060"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="00002060"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <color rgb="00660000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="00660000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -110,36 +51,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A9F5A9"/>
-        <bgColor rgb="00A9F5A9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A9D0F5"/>
-        <bgColor rgb="00A9D0F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5A9A9"/>
-        <bgColor rgb="00F5A9A9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
   </fills>
@@ -169,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -179,39 +90,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4455,1019 +4333,4 @@
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>The Monet 第1期 - 2座 销控网格图</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>总套数</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>在售 (Sale)</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>已定价未售</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>已售 (Sold)</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>暂停销售</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>待售 (Pending)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>28 套</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>28 套</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>楼层\房号</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="65" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>17/F</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="65" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>16/F</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="65" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>15/F</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>12/F</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="65" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>11/F</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="65" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>10/F</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="65" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>9/F</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="65" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>8/F</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>7/F</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="65" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>6/F</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="65" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>5/F</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="65" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>3/F</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="65" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2/F</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="65" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>1/F</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>The Monet 第1期 - 3座 销控网格图</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>总套数</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>在售 (Sale)</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>已定价未售</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>已售 (Sold)</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>暂停销售</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>待售 (Pending)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>45 套</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>45 套</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>楼层\房号</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="65" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>18/F</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="65" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>17/F</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="65" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>16/F</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>15/F</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="65" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>12/F</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="65" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>11/F</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="65" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>10/F</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="65" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>9/F</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>8/F</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="65" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>7/F</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="65" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>6/F</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="65" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>5/F</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="65" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>3/F</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="65" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>2/F</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="65" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>1/F</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>A | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>B | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>C | 暂无 (null房)
-暂无价格
-暂无呎价
-(待售)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>